<commit_message>
add example for Excel test list import
</commit_message>
<xml_diff>
--- a/harness/SemiATE_testlistimport.xlsx
+++ b/harness/SemiATE_testlistimport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jung\ATE\packages\envs\workonIssues\tb_semi_ate_example\harness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E32FAA7-11C0-4A9E-867A-E917E762D6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11801755-1A7D-4B8F-A740-BAE6499C103C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1770" yWindow="1320" windowWidth="24600" windowHeight="13020" xr2:uid="{6EC8AF89-4612-4129-A41E-2FE6FF877A00}"/>
+    <workbookView xWindow="-27885" yWindow="-15780" windowWidth="24660" windowHeight="12810" xr2:uid="{6EC8AF89-4612-4129-A41E-2FE6FF877A00}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
   <si>
     <t>Name</t>
   </si>
@@ -107,9 +107,6 @@
     <t>Offset</t>
   </si>
   <si>
-    <t>DAC test with offset, dnl + 14bit values</t>
-  </si>
-  <si>
     <t>dnl</t>
   </si>
   <si>
@@ -125,9 +122,6 @@
     <t>Contact Test only Pass/Fail Information</t>
   </si>
   <si>
-    <t>Contact Test  with output from Values</t>
-  </si>
-  <si>
     <t>Testlimit Low</t>
   </si>
   <si>
@@ -141,6 +135,22 @@
   </si>
   <si>
     <t>idd</t>
+  </si>
+  <si>
+    <t>DAC test with offset, dnl + 14bit values\nread all dac values</t>
+  </si>
+  <si>
+    <t>MPR</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Contact Test  with output from Values
+measure current</t>
   </si>
 </sst>
 </file>
@@ -185,10 +195,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -523,18 +536,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B5F5B7E-0213-440F-B769-C6BD1A0DCCF1}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="36.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -545,16 +558,16 @@
         <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>17</v>
@@ -563,13 +576,16 @@
         <v>18</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -588,11 +604,14 @@
       <c r="I2" t="s">
         <v>2</v>
       </c>
-      <c r="K2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>10020</v>
       </c>
@@ -608,8 +627,11 @@
       <c r="I3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>10025</v>
       </c>
@@ -625,8 +647,11 @@
       <c r="I4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -642,11 +667,14 @@
       <c r="F5">
         <v>99.1</v>
       </c>
-      <c r="K5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>10051</v>
       </c>
@@ -659,8 +687,11 @@
       <c r="F6">
         <v>900</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -679,11 +710,14 @@
       <c r="I7" t="s">
         <v>2</v>
       </c>
-      <c r="K7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>10101</v>
       </c>
@@ -699,8 +733,11 @@
       <c r="I8" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>10102</v>
       </c>
@@ -716,8 +753,11 @@
       <c r="I9" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>10103</v>
       </c>
@@ -733,16 +773,19 @@
       <c r="I10" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>21</v>
       </c>
       <c r="B11">
-        <v>10152</v>
+        <v>10150</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -751,15 +794,18 @@
         <v>4096</v>
       </c>
       <c r="J11" t="s">
-        <v>25</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="K11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12">
-        <v>10150</v>
+        <v>10151</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
@@ -779,13 +825,16 @@
       <c r="I12" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B13">
-        <v>10151</v>
+        <v>10152</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -793,13 +842,16 @@
       <c r="F13">
         <v>100</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B14">
-        <v>10152</v>
+        <v>10153</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E14">
         <v>6</v>
@@ -812,6 +864,9 @@
       </c>
       <c r="I14" t="s">
         <v>11</v>
+      </c>
+      <c r="J14" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>